<commit_message>
session 20260827 (cont.): prose chapters 4-6 redone twice (corrected to exclude inactive tables per researcher), cfg_prose_chapter retired + Prose.ps1 SetStatus built (#920), a real self-close-without-approval violation found and corrected into an approved resolution_kind gate design (#921 v2), bible_research/iba.db table reconciliation + physical-schema self-control (#922, found 3 unregistered iba.db tables), ch.2/ch.3 sections realigned to current stage terminology and CC+API/escalation collaboration model (#930/#932), prose change-log mechanism validated live against 949 rows (#931), full project-wide analytic-file census + multi-round consolidated raw-data/analytics folder design paused for researcher's own manual Explorer reorg (#929/#933) -- see session log for full detail, escalations #911-933
</commit_message>
<xml_diff>
--- a/iba/docs/escalation actions worksheet.xlsx
+++ b/iba/docs/escalation actions worksheet.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Bible_study_projects\iba\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D0D70A83-5955-4524-BE4A-C880A85FB3A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E091DE26-26FA-4A37-951E-39F1B79A41EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7AEB6694-A08E-49E1-807B-C60BA5639946}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Escalations" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="77">
   <si>
     <t>Escalation tool</t>
   </si>
@@ -243,7 +243,25 @@
     <t>DecisionRequired</t>
   </si>
   <si>
-    <r>
+    <t>AnswerRun|ResolveSelfCorrectable|EscalateToDecision</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00008B"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>on</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFA9A9A9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
       <t>-</t>
     </r>
     <r>
@@ -253,7 +271,135 @@
         <rFont val="Consolas"/>
         <family val="3"/>
       </rPr>
-      <t>RelatedActivity</t>
+      <t>hold</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFA9A9A9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>|</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00008B"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>in</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFA9A9A9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00008B"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>progress</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFA9A9A9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>|</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00008B"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>closed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFA9A9A9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>|</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00008B"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>withdraw</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFA9A9A9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>|</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00008B"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>supersede</t>
+    </r>
+  </si>
+  <si>
+    <t>review</t>
+  </si>
+  <si>
+    <t>revise</t>
+  </si>
+  <si>
+    <t>approval</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Issue</t>
+  </si>
+  <si>
+    <t>in-progress</t>
+  </si>
+  <si>
+    <t>supercede</t>
+  </si>
+  <si>
+    <t>supersede</t>
+  </si>
+  <si>
+    <t>reject</t>
+  </si>
+  <si>
+    <t>withdraw</t>
+  </si>
+  <si>
+    <t>hold</t>
+  </si>
+  <si>
+    <r>
+      <t>ready</t>
     </r>
     <r>
       <rPr>
@@ -262,16 +408,8 @@
         <rFont val="Consolas"/>
         <family val="3"/>
       </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <t>-FromID</t>
-  </si>
-  <si>
-    <t>AnswerRun|ResolveSelfCorrectable|EscalateToDecision</t>
-  </si>
-  <si>
+      <t>_</t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -279,7 +417,25 @@
         <rFont val="Consolas"/>
         <family val="3"/>
       </rPr>
-      <t>on</t>
+      <t>for</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00008B"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>approval</t>
     </r>
     <r>
       <rPr>
@@ -288,7 +444,7 @@
         <rFont val="Consolas"/>
         <family val="3"/>
       </rPr>
-      <t>-</t>
+      <t>|</t>
     </r>
     <r>
       <rPr>
@@ -297,7 +453,7 @@
         <rFont val="Consolas"/>
         <family val="3"/>
       </rPr>
-      <t>hold</t>
+      <t>approved</t>
     </r>
     <r>
       <rPr>
@@ -315,7 +471,7 @@
         <rFont val="Consolas"/>
         <family val="3"/>
       </rPr>
-      <t>in</t>
+      <t>reject</t>
     </r>
     <r>
       <rPr>
@@ -324,7 +480,7 @@
         <rFont val="Consolas"/>
         <family val="3"/>
       </rPr>
-      <t>-</t>
+      <t>|</t>
     </r>
     <r>
       <rPr>
@@ -333,7 +489,7 @@
         <rFont val="Consolas"/>
         <family val="3"/>
       </rPr>
-      <t>progress</t>
+      <t>revise</t>
     </r>
     <r>
       <rPr>
@@ -351,7 +507,7 @@
         <rFont val="Consolas"/>
         <family val="3"/>
       </rPr>
-      <t>closed</t>
+      <t>noted</t>
     </r>
     <r>
       <rPr>
@@ -369,188 +525,6 @@
         <rFont val="Consolas"/>
         <family val="3"/>
       </rPr>
-      <t>withdraw</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFA9A9A9"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>|</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00008B"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>supersede</t>
-    </r>
-  </si>
-  <si>
-    <t>review</t>
-  </si>
-  <si>
-    <t>revise</t>
-  </si>
-  <si>
-    <t>approval</t>
-  </si>
-  <si>
-    <t>Task</t>
-  </si>
-  <si>
-    <t>Issue</t>
-  </si>
-  <si>
-    <t>in-progress</t>
-  </si>
-  <si>
-    <t>supercede</t>
-  </si>
-  <si>
-    <t>supersede</t>
-  </si>
-  <si>
-    <t>reject</t>
-  </si>
-  <si>
-    <t>withdraw</t>
-  </si>
-  <si>
-    <t>hold</t>
-  </si>
-  <si>
-    <r>
-      <t>ready</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF333333"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00008B"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>for</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF333333"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00008B"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>approval</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFA9A9A9"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>|</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00008B"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>approved</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFA9A9A9"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>|</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00008B"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>reject</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFA9A9A9"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>|</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00008B"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>revise</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFA9A9A9"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>|</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00008B"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>noted</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFA9A9A9"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>|</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00008B"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
       <t>review|hold</t>
     </r>
   </si>
@@ -576,9 +550,6 @@
     <t>more info</t>
   </si>
   <si>
-    <t>Not related</t>
-  </si>
-  <si>
     <t>issue</t>
   </si>
   <si>
@@ -591,21 +562,9 @@
     <t>completed</t>
   </si>
   <si>
-    <t>This is a test</t>
-  </si>
-  <si>
-    <t>Escalation script testing</t>
-  </si>
-  <si>
-    <t>Set to revise</t>
-  </si>
-  <si>
     <t>Set to ready for approval</t>
   </si>
   <si>
-    <t>set to approved</t>
-  </si>
-  <si>
     <t>Resolution required</t>
   </si>
   <si>
@@ -618,16 +577,37 @@
     <t>Notice</t>
   </si>
   <si>
-    <t>set rejected and supersede</t>
-  </si>
-  <si>
     <t>-State</t>
   </si>
   <si>
-    <t>set to rejected</t>
-  </si>
-  <si>
     <t>set to on hold</t>
+  </si>
+  <si>
+    <t>substantial work has gone into governance, and I am not planning to do a another full sweep of governance</t>
+  </si>
+  <si>
+    <t>taken off hold.   Has this now been cleared</t>
+  </si>
+  <si>
+    <t>not approved, to be redesigned</t>
+  </si>
+  <si>
+    <t>Prose change log</t>
+  </si>
+  <si>
+    <t>Review prose change log to validate it is working correctly</t>
+  </si>
+  <si>
+    <t>section 69 update</t>
+  </si>
+  <si>
+    <t>Align the section  id 69 for programme with the current approach of using CC and API rather than AI and also work in how CC and Researcher is working in colaboration</t>
+  </si>
+  <si>
+    <t>Proceed with review and update</t>
+  </si>
+  <si>
+    <t>seems to be working</t>
   </si>
 </sst>
 </file>
@@ -693,7 +673,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -715,7 +695,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1050,13 +1029,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D0F6153-362F-416E-9FFC-C7AB60768AC1}">
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="31.85546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="29.28515625" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
     <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" style="2" customWidth="1"/>
     <col min="8" max="8" width="15.42578125" customWidth="1"/>
     <col min="10" max="10" width="14.7109375" customWidth="1"/>
     <col min="11" max="12" width="13" customWidth="1"/>
@@ -1064,22 +1044,22 @@
     <col min="14" max="14" width="22" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D4" t="s">
         <v>13</v>
@@ -1090,7 +1070,7 @@
       <c r="F4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="3" t="s">
         <v>29</v>
       </c>
       <c r="H4" s="1" t="s">
@@ -1106,7 +1086,7 @@
         <v>7</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>9</v>
@@ -1117,16 +1097,10 @@
       <c r="O4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="P4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:15" ht="90" x14ac:dyDescent="0.25">
       <c r="E5" s="1"/>
-      <c r="G5" t="s">
+      <c r="G5" s="2" t="s">
         <v>30</v>
       </c>
       <c r="H5" s="5" t="s">
@@ -1136,22 +1110,22 @@
         <v>32</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" ht="107.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="107.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C6" s="2" t="str">
-        <f>D6&amp;" " &amp;$E$4&amp;" "&amp;E6&amp;" "  &amp;$G$4&amp;" '"&amp;G6&amp;"' "&amp;$H$4&amp;" "&amp;H6&amp;" " &amp;$I$4&amp;" "&amp;I6&amp; " " &amp;$K$4 &amp; " " &amp;K6 &amp; " " &amp;$M$4&amp;" '" &amp; M6 &amp; "' " &amp;$N$4&amp;" '" &amp; N6 &amp;"' " &amp; $P$4 &amp; " '" &amp; P6 &amp; "' " &amp; $Q$4 &amp; " '"&amp;Q6&amp;"'"</f>
-        <v>iba\app\ps\Escalation.ps1 -action raise -Question 'title' -ResolutionKind DecisionRequired -Type issue -AssignedTo Researcher -Comment 'assigment' -Context 'more info' -RelatedActivity  'Not related' -FromID '-1'</v>
+        <f>D6&amp;" " &amp;$E$4&amp;" "&amp;E6&amp;" "  &amp;$G$4&amp;" '"&amp;G6&amp;"' "&amp;$H$4&amp;" "&amp;H6&amp;" " &amp;$I$4&amp;" "&amp;I6&amp; " " &amp;$K$4 &amp; " " &amp;K6 &amp; " " &amp;$M$4&amp;" '" &amp; M6 &amp; "' " &amp;$N$4&amp;" '" &amp; N6 &amp;"' "</f>
+        <v xml:space="preserve">iba\app\ps\Escalation.ps1 -action raise -Question 'Prose change log' -ResolutionKind DecisionRequired -Type issue -AssignedTo Researcher -Comment 'Review prose change log to validate it is working correctly' -Context 'more info' </v>
       </c>
       <c r="D6" t="s">
         <v>15</v>
@@ -1159,39 +1133,32 @@
       <c r="E6" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="9"/>
-      <c r="G6" s="4" t="s">
-        <v>56</v>
+      <c r="G6" s="8" t="s">
+        <v>71</v>
       </c>
       <c r="H6" t="s">
         <v>35</v>
       </c>
       <c r="I6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="K6" t="s">
         <v>25</v>
       </c>
       <c r="M6" s="8" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="N6" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="P6" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q6" s="4">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" ht="120" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="135" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C7" s="2" t="str">
-        <f>D7&amp;" " &amp;$E$4&amp;" "&amp;E7&amp;" "  &amp;$G$4&amp;" '"&amp;G7&amp;"' "&amp;$H$4&amp;" "&amp;H7&amp;" " &amp;$I$4&amp;" "&amp;I7&amp; " " &amp;$K$4 &amp; " " &amp;K7 &amp; " " &amp;$M$4&amp;" '" &amp; M7 &amp; "' " &amp;$N$4&amp;" '" &amp; N7 &amp;"' " &amp; $P$4 &amp; " '" &amp; P7 &amp; "' " &amp; $Q$4 &amp; " '"&amp;Q7&amp;"'"</f>
-        <v>iba\app\ps\Escalation.ps1 -action raise -Question 'title' -ResolutionKind DecisionRequired -Type task -AssignedTo Researcher -Comment 'assigment' -Context 'more info' -RelatedActivity  'Not related' -FromID '-1'</v>
+        <f>D7&amp;" " &amp;$E$4&amp;" "&amp;E7&amp;" "  &amp;$G$4&amp;" '"&amp;G7&amp;"' "&amp;$H$4&amp;" "&amp;H7&amp;" " &amp;$I$4&amp;" "&amp;I7&amp; " " &amp;$K$4 &amp; " " &amp;K7 &amp; " " &amp;$M$4&amp;" '" &amp; M7 &amp; "' " &amp;$N$4&amp;" '" &amp; N7 &amp;"' "</f>
+        <v xml:space="preserve">iba\app\ps\Escalation.ps1 -action raise -Question 'section 69 update' -ResolutionKind DecisionRequired -Type task -AssignedTo Researcher -Comment 'Align the section  id 69 for programme with the current approach of using CC and API rather than AI and also work in how CC and Researcher is working in colaboration' -Context '' </v>
       </c>
       <c r="D7" t="s">
         <v>15</v>
@@ -1199,39 +1166,30 @@
       <c r="E7" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="9"/>
-      <c r="G7" s="4" t="s">
-        <v>56</v>
+      <c r="G7" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="H7" t="s">
         <v>35</v>
       </c>
       <c r="I7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="K7" t="s">
         <v>25</v>
       </c>
       <c r="M7" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="N7" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="P7" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q7" s="4">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" ht="120" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+      <c r="N7" s="8"/>
+    </row>
+    <row r="8" spans="1:15" ht="90" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C8" s="2" t="str">
-        <f>D8&amp;" " &amp;$E$4&amp;" "&amp;E8&amp;" "  &amp;$G$4&amp;" '"&amp;G8&amp;"' "&amp;$H$4&amp;" "&amp;H8&amp;" " &amp;$I$4&amp;" "&amp;I8&amp; " " &amp;$K$4 &amp; " " &amp;K8 &amp; " " &amp;$M$4&amp;" '" &amp; M8 &amp; "' " &amp;$N$4&amp;" '" &amp; N8 &amp;"' " &amp; $P$4 &amp; " '" &amp; P8 &amp; "' " &amp; $Q$4 &amp; " '"&amp;Q8&amp;"'"</f>
-        <v>iba\app\ps\Escalation.ps1 -action raise -Question 'title' -ResolutionKind DecisionRequired -Type notice -AssignedTo Researcher -Comment 'assigment' -Context 'more info' -RelatedActivity  'Not related' -FromID '-1'</v>
+        <f>D8&amp;" " &amp;$E$4&amp;" "&amp;E8&amp;" "  &amp;$G$4&amp;" '"&amp;G8&amp;"' "&amp;$H$4&amp;" "&amp;H8&amp;" " &amp;$I$4&amp;" "&amp;I8&amp; " " &amp;$K$4 &amp; " " &amp;K8 &amp; " " &amp;$M$4&amp;" '" &amp; M8 &amp; "' " &amp;$N$4&amp;" '" &amp; N8 &amp;"' "</f>
+        <v xml:space="preserve">iba\app\ps\Escalation.ps1 -action raise -Question 'title' -ResolutionKind DecisionRequired -Type notice -AssignedTo Researcher -Comment 'assigment' -Context 'more info' </v>
       </c>
       <c r="D8" t="s">
         <v>15</v>
@@ -1239,285 +1197,266 @@
       <c r="E8" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="9"/>
-      <c r="G8" s="4" t="s">
-        <v>56</v>
+      <c r="G8" s="8" t="s">
+        <v>54</v>
       </c>
       <c r="H8" t="s">
         <v>35</v>
       </c>
       <c r="I8" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="K8" t="s">
         <v>25</v>
       </c>
       <c r="M8" s="8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="N8" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="P8" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q8" s="4">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-    </row>
-    <row r="11" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="105" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C11" s="2" t="str">
-        <f>D11&amp;" " &amp;$E$4&amp;" "&amp;E11&amp;" " &amp;$F$4&amp;" "&amp;F11&amp;" "  &amp;$G$4&amp;" '"&amp;G11&amp;"' " &amp;$J$4&amp;" "&amp;J11&amp; " " &amp;$K$4 &amp; " " &amp;K11 &amp; " " &amp;$M$4&amp;" '" &amp; M11 &amp; "' " &amp;$N$4&amp;" '" &amp; N11 &amp;"' " &amp; $P$4 &amp; " '" &amp; P11 &amp; "' " &amp; $Q$4 &amp; " '"&amp;Q11&amp;"'"</f>
-        <v>iba\app\ps\Escalation.ps1 -action update -Id 869 -Question '' -NextAction review -AssignedTo Claude -Comment 'This is a test' -Context 'Escalation script testing' -RelatedActivity  'Not related' -FromID '-1'</v>
+        <f>D11&amp;" " &amp;$E$4&amp;" "&amp;E11&amp;" " &amp;$F$4&amp;" "&amp;F11&amp;" "  &amp;$H$4&amp;" "&amp;H11&amp;" " &amp;$J$4&amp;" "&amp;J11&amp; " " &amp;$K$4 &amp; " " &amp;K11 &amp; " " &amp;$L$4 &amp; " " &amp;L11 &amp; " " &amp;$M$4&amp;" '" &amp; M11 &amp; "' " &amp;$N$4&amp;" '" &amp; N11 &amp;"' "</f>
+        <v xml:space="preserve">iba\app\ps\Escalation.ps1 -action update -Id 932 -ResolutionKind DecisionRequired -NextAction review -AssignedTo Claude -State in-progress -Comment 'Proceed with review and update' -Context '' </v>
       </c>
       <c r="D11" t="s">
         <v>15</v>
       </c>
       <c r="E11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F11" s="4">
-        <v>869</v>
+        <v>932</v>
+      </c>
+      <c r="H11" t="s">
+        <v>35</v>
       </c>
       <c r="J11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K11" t="s">
         <v>8</v>
       </c>
       <c r="L11" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="M11" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="N11" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="P11" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q11" s="4">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" ht="75" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="N11" s="8"/>
+    </row>
+    <row r="12" spans="1:15" ht="105" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C12" s="2" t="str">
-        <f>D12&amp;" " &amp;$E$4&amp;" "&amp;E12&amp;" " &amp;$F$4&amp;" "&amp;F12&amp;" "  &amp;$G$4&amp;" '"&amp;G12&amp;"' " &amp;$J$4&amp;" "&amp;J12&amp; " " &amp;$K$4 &amp; " " &amp;K12 &amp; " " &amp;$M$4&amp;" '" &amp; M12 &amp; "' " &amp;$N$4&amp;" '" &amp; N12 &amp;"' " &amp; $P$4 &amp; " '" &amp; P12 &amp; "' " &amp; $Q$4 &amp; " '"&amp;Q12&amp;"'"</f>
-        <v>iba\app\ps\Escalation.ps1 -action update -Id 869 -Question '' -NextAction revise -AssignedTo Claude -Comment 'Set to revise' -Context '' -RelatedActivity  '' -FromID ''</v>
+        <f>D12&amp;" " &amp;$E$4&amp;" "&amp;E12&amp;" " &amp;$F$4&amp;" "&amp;F12&amp;" "  &amp;$H$4&amp;" "&amp;H12&amp;" " &amp;$J$4&amp;" "&amp;J12&amp; " " &amp;$K$4 &amp; " " &amp;K12 &amp; " " &amp;$L$4 &amp; " " &amp;L12 &amp; " " &amp;$M$4&amp;" '" &amp; M12 &amp; "' " &amp;$N$4&amp;" '" &amp; N12 &amp;"' "</f>
+        <v xml:space="preserve">iba\app\ps\Escalation.ps1 -action update -Id 768 -ResolutionKind DecisionRequired -NextAction revise -AssignedTo Claude -State in-progress -Comment 'taken off hold.   Has this now been cleared' -Context '' </v>
       </c>
       <c r="D12" t="s">
         <v>15</v>
       </c>
       <c r="E12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F12" s="4">
-        <v>869</v>
+        <v>768</v>
+      </c>
+      <c r="H12" t="s">
+        <v>35</v>
       </c>
       <c r="J12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="K12" t="s">
         <v>8</v>
       </c>
       <c r="L12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="M12" s="8" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="N12" s="8"/>
-      <c r="P12" s="4"/>
-      <c r="Q12" s="4"/>
-    </row>
-    <row r="13" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:15" ht="120" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C13" s="2" t="str">
-        <f>D13&amp;" " &amp;$E$4&amp;" "&amp;E13&amp;" " &amp;$F$4&amp;" "&amp;F13&amp;" "  &amp;$G$4&amp;" '"&amp;G13&amp;"' " &amp;$J$4&amp;" "&amp;J13&amp; " " &amp;$K$4 &amp; " " &amp;K13 &amp; " " &amp;$M$4&amp;" '" &amp; M13 &amp; "' " &amp;$N$4&amp;" '" &amp; N13 &amp;"' " &amp;$O$4 &amp; " '"&amp; O13 &amp;"'" &amp; $P$4 &amp; " '" &amp; P13 &amp; "' " &amp; $Q$4 &amp; " '"&amp;Q13&amp;"'"</f>
-        <v>iba\app\ps\Escalation.ps1 -action update -Id 869 -Question '' -NextAction ready_for_approval -AssignedTo Researcher -Comment 'Set to ready for approval' -Context '' -Resolution 'Resolution required'-RelatedActivity  '' -FromID ''</v>
+        <f>D13&amp;" " &amp;$E$4&amp;" "&amp;E13&amp;" " &amp;$F$4&amp;" "&amp;F13&amp;" "  &amp;$H$4&amp;" "&amp;H13&amp;" " &amp;$J$4&amp;" "&amp;J13&amp; " " &amp;$K$4 &amp; " " &amp;K13 &amp; " "&amp;$L$4 &amp; " " &amp;L13 &amp; " " &amp;$M$4&amp;" '" &amp; M13 &amp; "' " &amp;$N$4&amp;" '" &amp; N13 &amp;"' " &amp;$O$4 &amp; " '"&amp; O13 &amp;"'"</f>
+        <v>iba\app\ps\Escalation.ps1 -action update -Id 921 -ResolutionKind DecisionRequired -NextAction ready_for_approval -AssignedTo Researcher -State in-progress -Comment 'Set to ready for approval' -Context '' -Resolution 'Resolution required'</v>
       </c>
       <c r="D13" t="s">
         <v>15</v>
       </c>
       <c r="E13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F13" s="4">
-        <v>869</v>
+        <v>921</v>
+      </c>
+      <c r="H13" t="s">
+        <v>35</v>
       </c>
       <c r="J13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="K13" t="s">
         <v>25</v>
       </c>
       <c r="L13" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="M13" s="8" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="N13" s="8"/>
       <c r="O13" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="P13" s="4"/>
-      <c r="Q13" s="4"/>
-    </row>
-    <row r="14" spans="1:17" ht="75" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="105" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C14" s="2" t="str">
-        <f>D14&amp;" " &amp;$E$4&amp;" "&amp;E14&amp;" " &amp;$F$4&amp;" "&amp;F14&amp;" "  &amp;$G$4&amp;" '"&amp;G14&amp;"' " &amp;$J$4&amp;" "&amp;J14&amp; " " &amp;$K$4 &amp; " " &amp;K14 &amp; " " &amp;$M$4&amp;" '" &amp; M14 &amp; "' " &amp;$N$4&amp;" '" &amp; N14 &amp;"' " &amp; $P$4 &amp; " '" &amp; P14 &amp; "' " &amp; $Q$4 &amp; " '"&amp;Q14&amp;"'"</f>
-        <v>iba\app\ps\Escalation.ps1 -action update -Id 869 -Question '' -NextAction approved -AssignedTo Researcher -Comment 'set to approved' -Context '' -RelatedActivity  '' -FromID ''</v>
+        <f>D14&amp;" " &amp;$E$4&amp;" "&amp;E14&amp;" " &amp;$F$4&amp;" "&amp;F14&amp;" "  &amp;$H$4&amp;" "&amp;H14&amp;" " &amp;$J$4&amp;" "&amp;J14&amp; " " &amp;$K$4 &amp; " " &amp;K14 &amp; " "&amp;$L$4 &amp; " " &amp;L14 &amp; " " &amp;$M$4&amp;" '" &amp; M14 &amp; "' " &amp;$N$4&amp;" '" &amp; N14 &amp;"' " &amp;$O$4 &amp; " '"&amp; O14 &amp;"'"</f>
+        <v>iba\app\ps\Escalation.ps1 -action update -Id 931 -ResolutionKind DecisionRequired -NextAction approved -AssignedTo Researcher -State completed -Comment 'seems to be working' -Context '' -Resolution ''</v>
       </c>
       <c r="D14" t="s">
         <v>15</v>
       </c>
       <c r="E14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F14" s="4">
-        <v>869</v>
+        <v>931</v>
+      </c>
+      <c r="H14" t="s">
+        <v>35</v>
       </c>
       <c r="J14" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="K14" t="s">
         <v>25</v>
       </c>
       <c r="L14" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="M14" s="8" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="N14" s="8"/>
-      <c r="P14" s="4"/>
-      <c r="Q14" s="4"/>
-    </row>
-    <row r="15" spans="1:17" ht="75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:15" ht="135" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2" t="str">
-        <f>D15&amp;" " &amp;$E$4&amp;" "&amp;E15&amp;" " &amp;$F$4&amp;" "&amp;F15&amp;" "  &amp;$G$4&amp;" '"&amp;G15&amp;"' " &amp;$J$4&amp;" "&amp;J15&amp; " " &amp;$K$4 &amp; " " &amp;K15 &amp; " "&amp; $L$4 &amp; " " &amp;L15 &amp;" "  &amp;$M$4&amp;" '" &amp; M15 &amp; "' " &amp;$N$4&amp;" '" &amp; N15 &amp;"' " &amp; $P$4 &amp; " '" &amp; P15 &amp; "' " &amp; $Q$4 &amp; " '"&amp;Q15&amp;"'"</f>
-        <v>iba\app\ps\Escalation.ps1 -action update -Id 870 -Question '' -NextAction reject -AssignedTo Claude -State supersede -Comment 'set rejected and supersede' -Context '' -RelatedActivity  '' -FromID ''</v>
+        <f>D15&amp;" " &amp;$E$4&amp;" "&amp;E15&amp;" " &amp;$F$4&amp;" "&amp;F15&amp;" "  &amp;$H$4&amp;" "&amp;H15&amp;" " &amp;$J$4&amp;" "&amp;J15&amp; " " &amp;$K$4 &amp; " " &amp;K15 &amp; " "&amp;$L$4 &amp; " " &amp;L15 &amp; " " &amp;$M$4&amp;" '" &amp; M15 &amp; "' " &amp;$N$4&amp;" '" &amp; N15 &amp;"' " &amp;$O$4 &amp; " '"&amp; O15 &amp;"'"</f>
+        <v>iba\app\ps\Escalation.ps1 -action update -Id 9 -ResolutionKind  -NextAction reject -AssignedTo Claude -State supersede -Comment 'substantial work has gone into governance, and I am not planning to do a another full sweep of governance' -Context '' -Resolution ''</v>
       </c>
       <c r="D15" t="s">
         <v>15</v>
       </c>
       <c r="E15" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F15" s="4">
-        <v>870</v>
+        <v>9</v>
       </c>
       <c r="J15" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K15" t="s">
         <v>8</v>
       </c>
       <c r="L15" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="M15" s="8" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="N15" s="8"/>
-      <c r="P15" s="4"/>
-      <c r="Q15" s="4"/>
-    </row>
-    <row r="16" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:15" ht="105" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C16" s="2" t="str">
-        <f>D16&amp;" " &amp;$E$4&amp;" "&amp;E16&amp;" " &amp;$F$4&amp;" "&amp;F16&amp;" "  &amp;$G$4&amp;" '"&amp;G16&amp;"' " &amp;$J$4&amp;" "&amp;J16&amp; " " &amp;$K$4 &amp; " " &amp;K16 &amp; " "&amp; $L$4 &amp; " " &amp;L16 &amp;" "  &amp;$M$4&amp;" '" &amp; M16 &amp; "' " &amp;$N$4&amp;" '" &amp; N16 &amp;"' " &amp; $P$4 &amp; " '" &amp; P16 &amp; "' " &amp; $Q$4 &amp; " '"&amp;Q16&amp;"'"</f>
-        <v>iba\app\ps\Escalation.ps1 -action update -Id 873 -Question '' -NextAction reject -AssignedTo Claude -State withdraw -Comment 'set to rejected' -Context '' -RelatedActivity  '' -FromID ''</v>
+        <f>D16&amp;" " &amp;$E$4&amp;" "&amp;E16&amp;" " &amp;$F$4&amp;" "&amp;F16&amp;" "  &amp;$H$4&amp;" "&amp;H16&amp;" " &amp;$J$4&amp;" "&amp;J16&amp; " " &amp;$K$4 &amp; " " &amp;K16 &amp; " "&amp;$L$4 &amp; " " &amp;L16 &amp; " " &amp;$M$4&amp;" '" &amp; M16 &amp; "' " &amp;$N$4&amp;" '" &amp; N16 &amp;"' " &amp;$O$4 &amp; " '"&amp; O16 &amp;"'"</f>
+        <v>iba\app\ps\Escalation.ps1 -action update -Id 912 -ResolutionKind  -NextAction reject -AssignedTo Claude -State withdraw -Comment 'not approved, to be redesigned' -Context '' -Resolution ''</v>
       </c>
       <c r="D16" t="s">
         <v>15</v>
       </c>
       <c r="E16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F16" s="4">
-        <v>873</v>
+        <v>912</v>
       </c>
       <c r="J16" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K16" t="s">
         <v>8</v>
       </c>
       <c r="L16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="M16" s="8" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="N16" s="8"/>
-      <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
-    </row>
-    <row r="17" spans="1:17" ht="90" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:15" ht="90" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C17" s="2" t="str">
-        <f>D17&amp;" " &amp;$E$4&amp;" "&amp;E17&amp;" " &amp;$F$4&amp;" "&amp;F17&amp;" "  &amp;$G$4&amp;" '"&amp;G17&amp;"' " &amp;$K$4 &amp; " " &amp;K17&amp; " "&amp;$L$4 &amp; " " &amp;L17 &amp; " " &amp;$M$4&amp;" '" &amp; M17 &amp; "' " &amp;$N$4&amp;" '" &amp; N17 &amp;"' " &amp; $P$4 &amp; " '" &amp; P17 &amp; "' " &amp; $Q$4 &amp; " '"&amp;Q17&amp;"'"</f>
-        <v>iba\app\ps\Escalation.ps1 -action update -Id 874 -Question '' -AssignedTo Researcher -State on-hold -Comment 'set to on hold' -Context '' -RelatedActivity  '' -FromID ''</v>
+        <f>D17&amp;" " &amp;$E$4&amp;" "&amp;E17&amp;" " &amp;$F$4&amp;" "&amp;F17&amp;" "  &amp;$H$4&amp;" "&amp;H17&amp;" " &amp;$J$4&amp;" "&amp;J17&amp; " " &amp;$K$4 &amp; " " &amp;K17 &amp; " "&amp;$L$4 &amp; " " &amp;L17 &amp; " " &amp;$M$4&amp;" '" &amp; M17 &amp; "' " &amp;$N$4&amp;" '" &amp; N17 &amp;"' " &amp;$O$4 &amp; " '"&amp; O17 &amp;"'"</f>
+        <v>iba\app\ps\Escalation.ps1 -action update -Id 874 -ResolutionKind  -NextAction revise -AssignedTo Researcher -State on-hold -Comment 'set to on hold' -Context '' -Resolution ''</v>
       </c>
       <c r="D17" t="s">
         <v>15</v>
       </c>
       <c r="E17" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F17" s="4">
         <v>874</v>
       </c>
       <c r="J17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="K17" t="s">
         <v>25</v>
       </c>
       <c r="L17" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="M17" s="8" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="N17" s="8"/>
-      <c r="P17" s="4"/>
-      <c r="Q17" s="4"/>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -1535,7 +1474,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="23" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>18</v>
       </c>
@@ -1550,12 +1489,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>12</v>
       </c>
@@ -1571,7 +1510,7 @@
       <c r="F27" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G27" s="1"/>
+      <c r="G27" s="3"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1" t="s">
@@ -1588,15 +1527,15 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="E28" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J28" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>21</v>
       </c>

</xml_diff>

<commit_message>
session 20260828 (cont.): PS tools workbook built, M08 cluster-work pilot (#1005) complete, windows-debate reopened, escalation #1006 raised for tomorrow
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iba/docs/escalation actions worksheet.xlsx
+++ b/iba/docs/escalation actions worksheet.xlsx
@@ -379,13 +379,13 @@
     <t>Task</t>
   </si>
   <si>
-    <t>section 69 update</t>
+    <t>Explore existing cluster work</t>
   </si>
   <si>
     <t>task</t>
   </si>
   <si>
-    <t>Align the section  id 69 for programme with the current approach of using CC and API rather than AI and also work in how CC and Researcher is working in colaboration</t>
+    <t>The objective is to explore and assess the existing cluster work to determine how much, and in what format can it be harvested and augmented to complete the cluster analysis</t>
   </si>
   <si>
     <t>Notice</t>
@@ -415,7 +415,7 @@
     <t>in-progress</t>
   </si>
   <si>
-    <t>proceed to prepare for approval</t>
+    <t>the initial assesment will be on M08 C:\Bible_study_projects\_analytics\clusters\M08-Pride start off by summarising what is in the folder and extract everything from the DB about M08.  all files must go back on this folder, not in another place.</t>
   </si>
   <si>
     <t>revise</t>
@@ -1220,7 +1220,7 @@
         <v>31</v>
       </c>
       <c r="C7" s="10">
-        <f>D7&amp;" " &amp;$E$4&amp;" "&amp;E7&amp;" "  &amp;$G$4&amp;" '"&amp;G7&amp;"' "&amp;$H$4&amp;" "&amp;H7&amp;" " &amp;$I$4&amp;" "&amp;I7&amp; " " &amp;$K$4 &amp; " " &amp;K7 &amp; " " &amp;$M$4&amp;" '" &amp; M7 &amp; "' " &amp;$N$4&amp;" '" &amp; N7 &amp;"' "</f>
+        <f>D7&amp;" " &amp;$E$4&amp;" "&amp;E7&amp;" "  &amp;$G$4&amp;" ' "&amp;G7&amp;" ' "&amp;$H$4&amp;" "&amp;H7&amp;" " &amp;$I$4&amp;" "&amp;I7&amp; " " &amp;$K$4 &amp; " " &amp;K7 &amp; " " &amp;$M$4&amp;" ' " &amp; M7 &amp; " ' " &amp;$N$4&amp;" ' " &amp; N7 &amp;" ' "</f>
       </c>
       <c r="D7" s="2" t="s">
         <v>23</v>
@@ -1328,7 +1328,7 @@
         <v>40</v>
       </c>
       <c r="C11" s="10">
-        <f>D11&amp;" " &amp;$E$4&amp;" "&amp;E11&amp;" " &amp;$F$4&amp;" "&amp;F11&amp;" "  &amp;$H$4&amp;" "&amp;H11&amp;" " &amp;$J$4&amp;" "&amp;J11&amp; " " &amp;$K$4 &amp; " " &amp;K11 &amp; " " &amp;$L$4 &amp; " " &amp;L11 &amp; " " &amp;$M$4&amp;" '" &amp; M11 &amp; "' " &amp;$N$4&amp;" '" &amp; N11 &amp;"' "</f>
+        <f>D11&amp;" " &amp;$E$4&amp;" "&amp;E11&amp;" " &amp;$F$4&amp;" "&amp;F11&amp;" "  &amp;$H$4&amp;" "&amp;H11&amp;" " &amp;$J$4&amp;" "&amp;J11&amp; " " &amp;$K$4 &amp; " " &amp;K11 &amp; " " &amp;$L$4 &amp; " " &amp;L11 &amp; " " &amp;$M$4&amp;" ' " &amp; M11 &amp; " ' " &amp;$N$4&amp;" ' " &amp; N11 &amp;" ' "</f>
       </c>
       <c r="D11" s="1" t="s">
         <v>23</v>
@@ -1337,7 +1337,7 @@
         <v>41</v>
       </c>
       <c r="F11" s="12">
-        <v>935</v>
+        <v>1005</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2" t="s">

</xml_diff>